<commit_message>
feat: publish AI-first infographic courseware v12
</commit_message>
<xml_diff>
--- a/activities/Activity-01-Decode-a-Customer-Survey-Infographic/A01-Decode-a-Customer-Survey-Infographic-Data.xlsx
+++ b/activities/Activity-01-Decode-a-Customer-Survey-Infographic/A01-Decode-a-Customer-Survey-Infographic-Data.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Analysis" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Source Notes" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="AI Prompt Lab" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Data!$A$1:$D$5</definedName>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
   <si>
     <t xml:space="preserve">Segment</t>
   </si>
@@ -57,22 +58,13 @@
     <t xml:space="preserve">Row count</t>
   </si>
   <si>
-    <t xml:space="preserve">Average Responses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Responses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Average SatisfactionPct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total SatisfactionPct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Average AppUserPct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total AppUserPct</t>
+    <t xml:space="preserve">Total responses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted satisfaction pct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weighted app-user pct</t>
   </si>
   <si>
     <t xml:space="preserve">Decision note</t>
@@ -96,7 +88,7 @@
     <t xml:space="preserve">Activity</t>
   </si>
   <si>
-    <t xml:space="preserve">01 - Decode a Customer Survey Infographic</t>
+    <t xml:space="preserve">01 - Use AI to Clean Data and Extract Insights</t>
   </si>
   <si>
     <t xml:space="preserve">Data status</t>
@@ -108,13 +100,67 @@
     <t xml:space="preserve">Generated</t>
   </si>
   <si>
-    <t xml:space="preserve">15 August 2026</t>
+    <t xml:space="preserve">16 August 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Owner</t>
   </si>
   <si>
     <t xml:space="preserve">Learner working copy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prompt stage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copy-ready prompt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Output verification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewer / owner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data analyst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Using only the attached approved sources, create a source register, identify duplicates or conflicting definitions, clean the table, show formulas or transformations, and return five candidate insights with citations, caveats and a confidence note. Do not invent missing values.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter approved sources</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter checks performed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter edits made</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infographic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a one-page executive infographic for Singapore retail managers. Lead with one decision insight, show three supporting metrics, include a five-stage flow and a source footer. Use a clean professional style, strong hierarchy and no invented data. Leave critical labels editable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Text to image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a clean vector-like sustainability delivery illustration for a PowerPoint infographic: one electric van, one reusable parcel, a simple route and a feedback symbol. Transparent background, consistent blue/teal/violet/amber palette, no text, no logo, no watermark.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gemini Notebook deck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create Presenter Slides for business stakeholders. Focus on the verified decision insight, use a concise professional style, include source-grounded comparisons and a final recommendation. Avoid claims not supported by selected sources. Download PowerPoint when available; otherwise download PDF and identify what must be rebuilt as editable native PowerPoint objects.</t>
   </si>
 </sst>
 </file>
@@ -124,7 +170,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -176,8 +222,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -194,6 +246,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7C3AED"/>
+        <bgColor rgb="FF993366"/>
       </patternFill>
     </fill>
   </fills>
@@ -240,7 +298,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -271,6 +329,14 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -371,7 +437,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF7C3AED"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -698,8 +764,8 @@
         <v>10</v>
       </c>
       <c r="B5" s="0" t="n">
-        <f aca="false">IFERROR(AVERAGE(Data!B2:B5),0)</f>
-        <v>105</v>
+        <f aca="false">SUM(Data!B2:B5)</f>
+        <v>420</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -707,8 +773,8 @@
         <v>11</v>
       </c>
       <c r="B6" s="0" t="n">
-        <f aca="false">SUM(Data!B2:B5)</f>
-        <v>420</v>
+        <f aca="false">IFERROR(SUMPRODUCT(Data!B2:B5,Data!C2:C5)/SUM(Data!B2:B5),0)</f>
+        <v>77.8095238095238</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -716,36 +782,18 @@
         <v>12</v>
       </c>
       <c r="B7" s="0" t="n">
-        <f aca="false">IFERROR(AVERAGE(Data!C2:C5),0)</f>
-        <v>75.75</v>
+        <f aca="false">IFERROR(SUMPRODUCT(Data!B2:B5,Data!D2:D5)/SUM(Data!B2:B5),0)</f>
+        <v>59.8809523809524</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="0" t="n">
-        <f aca="false">SUM(Data!C2:C5)</f>
-        <v>303</v>
-      </c>
+      <c r="A8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="0" t="n">
-        <f aca="false">IFERROR(AVERAGE(Data!D2:D5),0)</f>
-        <v>51.75</v>
-      </c>
+      <c r="A9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="0" t="n">
-        <f aca="false">SUM(Data!D2:D5)</f>
-        <v>207</v>
-      </c>
+      <c r="A10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4"/>
@@ -761,10 +809,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -792,50 +840,176 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="C1" s="8" t="s">
         <v>29</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>